<commit_message>
Foulane Adventures : désignation de référencement sur la fiche technique et la matrice
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/foulaneavT1-T2_kit/fiche-technique-matrice.xlsx
+++ b/foulaneavT1-T2_kit/fiche-technique-matrice.xlsx
@@ -19,10 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.00 &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -1536,12 +1535,12 @@
     <row r="2" ht="110" customHeight="1">
       <c r="A2" s="91" t="inlineStr">
         <is>
-          <t>Foulane Adventures - Tome 1 : Les filets fantômes</t>
+          <t>Foulane Adventures "Les filets fantômes" - tome 1</t>
         </is>
       </c>
       <c r="B2" s="91" t="inlineStr">
         <is>
-          <t>La Famille Foulane en comics</t>
+          <t>Les filets fantômes</t>
         </is>
       </c>
       <c r="C2" s="92" t="inlineStr">
@@ -1682,12 +1681,12 @@
     <row r="3" ht="110" customHeight="1">
       <c r="A3" s="91" t="inlineStr">
         <is>
-          <t>Foulane Adventures - Tome 2 : L'or du mont Botak</t>
+          <t>Foulane Adventures "L'or du mont Botak" - tome 2</t>
         </is>
       </c>
       <c r="B3" s="91" t="inlineStr">
         <is>
-          <t>La Famille Foulane en comics</t>
+          <t>L'or du mont Botak</t>
         </is>
       </c>
       <c r="C3" s="92" t="inlineStr">
@@ -4441,7 +4440,7 @@
     <col width="11.42578125" customWidth="1" min="4" max="4"/>
     <col width="11.42578125" customWidth="1" style="53" min="13" max="13"/>
     <col hidden="1" width="24.85546875" customWidth="1" style="53" min="14" max="14"/>
-    <col hidden="1" style="53" min="15" max="19"/>
+    <col hidden="1" width="13" customWidth="1" style="53" min="15" max="19"/>
     <col width="11.42578125" customWidth="1" style="53" min="20" max="23"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Kit Foulane Adventures : EAN T1 9782919843992, prix 11,50 €, 4es à jour
</commit_message>
<xml_diff>
--- a/foulaneavT1-T2_kit/fiche-technique-matrice.xlsx
+++ b/foulaneavT1-T2_kit/fiche-technique-matrice.xlsx
@@ -675,7 +675,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -924,6 +924,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1545,7 +1548,7 @@
       </c>
       <c r="C2" s="92" t="inlineStr">
         <is>
-          <t>9789998770607</t>
+          <t>9782919843992</t>
         </is>
       </c>
       <c r="D2" s="91" t="inlineStr">
@@ -1559,7 +1562,7 @@
         <v>9.478673000000001</v>
       </c>
       <c r="F2" s="94" t="n">
-        <v>10</v>
+        <v>11.5</v>
       </c>
       <c r="G2" s="91" t="inlineStr">
         <is>
@@ -1705,7 +1708,7 @@
         <v>9.478673000000001</v>
       </c>
       <c r="F3" s="94" t="n">
-        <v>10</v>
+        <v>11.5</v>
       </c>
       <c r="G3" s="91" t="inlineStr">
         <is>
@@ -4340,7 +4343,7 @@
       </c>
       <c r="B8" s="37" t="inlineStr">
         <is>
-          <t>10 € TTC, prix imprimé sur la couverture.</t>
+          <t>11,50 € TTC pour les deux tomes, prix imprimé sur les 4es (confirmé le 28/09).</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4357,7 +4360,7 @@
       </c>
       <c r="B9" s="37" t="inlineStr">
         <is>
-          <t>Lus sur les codes-barres imprimés : T1 9789998770607, T2 9782919843220.</t>
+          <t>T1 9782919843992 (4e de couverture à jour, 28/09 ; l'ancien 9789998770607 était faux). T2 9782919843220 lu sur le code-barres imprimé.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">

</xml_diff>